<commit_message>
docs(core): clarify autofilter limits in examples
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
+++ b/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
@@ -4,6 +4,7 @@
   <sheets>
     <sheet name="Kitchen Sink Grid" sheetId="1" r:id="rId1"/>
     <sheet name="RTL Review" sheetId="2" r:id="rId2"/>
+    <sheet name="Filtered Review" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -1396,4 +1397,376 @@
     <mergeCell ref="M4:M6"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="29" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
+    <col min="12" max="12" width="42" customWidth="1"/>
+    <col min="13" max="13" width="27" customWidth="1"/>
+  </cols>
+  <autoFilter ref="A1:M10"/>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="4">
+        <v>8</v>
+      </c>
+      <c r="H2" s="5">
+        <v>1450</v>
+      </c>
+      <c r="I2" s="6">
+        <v>11600</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" s="9">
+        <v>45719.395833333336</v>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="4">
+        <v>1</v>
+      </c>
+      <c r="H3" s="5">
+        <v>950</v>
+      </c>
+      <c r="I3" s="10">
+        <v>950</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="8"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="4">
+        <v>24</v>
+      </c>
+      <c r="H4" s="5">
+        <v>79</v>
+      </c>
+      <c r="I4" s="6">
+        <v>1896</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M4" s="9">
+        <v>45723.395833333336</v>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="4">
+        <v>2</v>
+      </c>
+      <c r="H5" s="5">
+        <v>1250</v>
+      </c>
+      <c r="I5" s="6">
+        <v>2500</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" s="8"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="4">
+        <v>1</v>
+      </c>
+      <c r="H6" s="5">
+        <v>600</v>
+      </c>
+      <c r="I6" s="10">
+        <v>600</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="8"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="9"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="4">
+        <v>5</v>
+      </c>
+      <c r="H7" s="5">
+        <v>39</v>
+      </c>
+      <c r="I7" s="6">
+        <v>195</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M7" s="9">
+        <v>45728.395833333336</v>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="4">
+        <v>14</v>
+      </c>
+      <c r="H8" s="5">
+        <v>520</v>
+      </c>
+      <c r="I8" s="6">
+        <v>7280</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" s="9">
+        <v>45734.395833333336</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="4">
+        <v>2</v>
+      </c>
+      <c r="H9" s="5">
+        <v>2100</v>
+      </c>
+      <c r="I9" s="6">
+        <v>4200</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" s="8"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="9"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="12">
+        <v>4</v>
+      </c>
+      <c r="G10" s="12">
+        <v>57</v>
+      </c>
+      <c r="I10" s="13">
+        <v>29221</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="K4:K6"/>
+    <mergeCell ref="L4:L6"/>
+    <mergeCell ref="M4:M6"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="M8:M9"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(core): disable autofilter on merged report rows
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
+++ b/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
@@ -1401,24 +1401,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
     <col min="4" max="4" width="29" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="32" customWidth="1"/>
-    <col min="12" max="12" width="42" customWidth="1"/>
-    <col min="13" max="13" width="27" customWidth="1"/>
+    <col min="5" max="5" width="32" customWidth="1"/>
+    <col min="6" max="6" width="42" customWidth="1"/>
+    <col min="7" max="7" width="27" customWidth="1"/>
   </cols>
-  <autoFilter ref="A1:M10"/>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
@@ -1434,30 +1427,12 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1474,299 +1449,91 @@
       <c r="D2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="4">
-        <v>8</v>
-      </c>
-      <c r="H2" s="5">
-        <v>1450</v>
-      </c>
-      <c r="I2" s="6">
-        <v>11600</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" s="8" t="s">
+      <c r="E2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="9">
+      <c r="G2" s="9">
         <v>45719.395833333336</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="4">
-        <v>1</v>
-      </c>
-      <c r="H3" s="5">
-        <v>950</v>
-      </c>
-      <c r="I3" s="10">
-        <v>950</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="8"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="9"/>
+      <c r="A3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="9">
+        <v>45723.395833333336</v>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="4">
-        <v>24</v>
-      </c>
-      <c r="H4" s="5">
-        <v>79</v>
-      </c>
-      <c r="I4" s="6">
-        <v>1896</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="M4" s="9">
-        <v>45723.395833333336</v>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" s="4">
-        <v>2</v>
-      </c>
-      <c r="H5" s="5">
-        <v>1250</v>
-      </c>
-      <c r="I5" s="6">
-        <v>2500</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" s="8"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="9"/>
-    </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="4">
-        <v>1</v>
-      </c>
-      <c r="H6" s="5">
-        <v>600</v>
-      </c>
-      <c r="I6" s="10">
-        <v>600</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="K6" s="8"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="9"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="4">
-        <v>5</v>
-      </c>
-      <c r="H7" s="5">
-        <v>39</v>
-      </c>
-      <c r="I7" s="6">
-        <v>195</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M7" s="9">
+      <c r="G4" s="9">
         <v>45728.395833333336</v>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="2" t="s">
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="4">
-        <v>14</v>
-      </c>
-      <c r="H8" s="5">
-        <v>520</v>
-      </c>
-      <c r="I8" s="6">
-        <v>7280</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="M8" s="9">
+      <c r="G5" s="9">
         <v>45734.395833333336</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="4">
-        <v>2</v>
-      </c>
-      <c r="H9" s="5">
-        <v>2100</v>
-      </c>
-      <c r="I9" s="6">
-        <v>4200</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" s="8"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="9"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="12">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="12">
         <v>4</v>
       </c>
-      <c r="G10" s="12">
-        <v>57</v>
-      </c>
-      <c r="I10" s="13">
-        <v>29221</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="K4:K6"/>
-    <mergeCell ref="L4:L6"/>
-    <mergeCell ref="M4:M6"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
-  </mergeCells>
+  <autoFilter ref="A1:G6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(core): add formula summaries to kitchen sink
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
+++ b/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
@@ -5,12 +5,13 @@
     <sheet name="Kitchen Sink Grid" sheetId="1" r:id="rId1"/>
     <sheet name="RTL Review" sheetId="2" r:id="rId2"/>
     <sheet name="Filtered Review" sheetId="3" r:id="rId3"/>
+    <sheet name="Formula Summaries" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>Order</t>
   </si>
@@ -176,6 +177,12 @@
   </si>
   <si>
     <t>Network gateway</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
@@ -1536,4 +1543,84 @@
   </sheetData>
   <autoFilter ref="A1:G6"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="5">
+        <v>12550</v>
+      </c>
+      <c r="C2" s="9">
+        <v>45719.395833333336</v>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5">
+        <v>4996</v>
+      </c>
+      <c r="C3" s="9">
+        <v>45723.395833333336</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="5">
+        <v>195</v>
+      </c>
+      <c r="C4" s="9">
+        <v>45728.395833333336</v>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="5">
+        <v>11480</v>
+      </c>
+      <c r="C5" s="9">
+        <v>45734.395833333336</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="13">
+        <f>SUM(B2:B5)</f>
+      </c>
+      <c r="C6" s="12">
+        <f>MAX(C2:C5)</f>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(core): inherit column formatting for formula summaries
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
+++ b/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
@@ -291,7 +291,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -331,6 +331,9 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1617,7 +1620,7 @@
       <c r="B6" s="13">
         <f>SUM(B2:B5)</f>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="14">
         <f>MAX(C2:C5)</f>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(core): add typed formula column DSL
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
+++ b/packages/typed-xlsx/examples/kitchen-sink-buffered.xlsx
@@ -6,12 +6,13 @@
     <sheet name="RTL Review" sheetId="2" r:id="rId2"/>
     <sheet name="Filtered Review" sheetId="3" r:id="rId3"/>
     <sheet name="Formula Summaries" sheetId="4" r:id="rId4"/>
+    <sheet name="Formula Columns" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Order</t>
   </si>
@@ -182,16 +183,48 @@
     <t>Amount</t>
   </si>
   <si>
+    <t>Items</t>
+  </si>
+  <si>
+    <t>Fulfilled %</t>
+  </si>
+  <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>AVERAGE / LATEST</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>Activated</t>
+  </si>
+  <si>
+    <t>Gross</t>
+  </si>
+  <si>
+    <t>Net</t>
+  </si>
+  <si>
+    <t>Utilization</t>
+  </si>
+  <si>
+    <t>Segment</t>
+  </si>
+  <si>
+    <t>Risk</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0%"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -291,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -332,8 +365,20 @@
     <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1550,12 +1595,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1566,6 +1613,12 @@
         <v>54</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1576,7 +1629,13 @@
       <c r="B2" s="5">
         <v>12550</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="E2" s="9">
         <v>45719.395833333336</v>
       </c>
     </row>
@@ -1587,7 +1646,13 @@
       <c r="B3" s="5">
         <v>4996</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="4">
+        <v>3</v>
+      </c>
+      <c r="D3" s="14">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="E3" s="9">
         <v>45723.395833333336</v>
       </c>
     </row>
@@ -1598,7 +1663,13 @@
       <c r="B4" s="5">
         <v>195</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="14">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9">
         <v>45728.395833333336</v>
       </c>
     </row>
@@ -1609,19 +1680,235 @@
       <c r="B5" s="5">
         <v>11480</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="14">
+        <v>1</v>
+      </c>
+      <c r="E5" s="9">
         <v>45734.395833333336</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="13">
-        <f>SUM(B2:B5)</f>
-      </c>
-      <c r="C6" s="14">
-        <f>MAX(C2:C5)</f>
+        <f>ROUND(SUM(B2:B5),2)</f>
+      </c>
+      <c r="C6" s="15">
+        <f>SUM(C2:C5)</f>
+      </c>
+      <c r="D6" s="16">
+        <f>ROUND(AVERAGE(D2:D5),4)</f>
+      </c>
+      <c r="E6" s="12"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="13">
+        <f>ROUND(AVERAGE(B2:B5),2)</f>
+      </c>
+      <c r="C7" s="15">
+        <f>AVERAGE(C2:C5)</f>
+      </c>
+      <c r="D7" s="16">
+        <f>MAX(MAX(D2:D5),0)</f>
+      </c>
+      <c r="E7" s="17">
+        <f>MAX(MAX(E2:E5),0)</f>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="4">
+        <v>9</v>
+      </c>
+      <c r="C2" s="5">
+        <v>1200</v>
+      </c>
+      <c r="D2" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="E2" s="4">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5">
+        <f>ROUND((B2*C2),2)</f>
+      </c>
+      <c r="G2" s="5">
+        <f>ROUND((F2*(1-D2)),2)</f>
+      </c>
+      <c r="H2" s="14">
+        <f>IF((B2&gt;0),ROUND((E2/B2),4),0)</f>
+      </c>
+      <c r="I2" s="2">
+        <f>IF(OR((G2&gt;=5000),(H2&gt;=0.85)),"HIGH",IF((D2&gt;=0.15),"WATCH","STANDARD"))</f>
+      </c>
+      <c r="J2" s="2">
+        <f>IF(OR((I2="WATCH"),(H2&lt;0.5)),"REVIEW","OK")</f>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="4">
+        <v>27</v>
+      </c>
+      <c r="C3" s="5">
+        <v>643</v>
+      </c>
+      <c r="D3" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="E3" s="4">
+        <v>26</v>
+      </c>
+      <c r="F3" s="5">
+        <f>ROUND((B3*C3),2)</f>
+      </c>
+      <c r="G3" s="5">
+        <f>ROUND((F3*(1-D3)),2)</f>
+      </c>
+      <c r="H3" s="14">
+        <f>IF((B3&gt;0),ROUND((E3/B3),4),0)</f>
+      </c>
+      <c r="I3" s="2">
+        <f>IF(OR((G3&gt;=5000),(H3&gt;=0.85)),"HIGH",IF((D3&gt;=0.15),"WATCH","STANDARD"))</f>
+      </c>
+      <c r="J3" s="2">
+        <f>IF(OR((I3="WATCH"),(H3&lt;0.5)),"REVIEW","OK")</f>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="4">
+        <v>5</v>
+      </c>
+      <c r="C4" s="5">
+        <v>39</v>
+      </c>
+      <c r="D4" s="18">
+        <v>0.03</v>
+      </c>
+      <c r="E4" s="4">
+        <v>5</v>
+      </c>
+      <c r="F4" s="5">
+        <f>ROUND((B4*C4),2)</f>
+      </c>
+      <c r="G4" s="5">
+        <f>ROUND((F4*(1-D4)),2)</f>
+      </c>
+      <c r="H4" s="14">
+        <f>IF((B4&gt;0),ROUND((E4/B4),4),0)</f>
+      </c>
+      <c r="I4" s="2">
+        <f>IF(OR((G4&gt;=5000),(H4&gt;=0.85)),"HIGH",IF((D4&gt;=0.15),"WATCH","STANDARD"))</f>
+      </c>
+      <c r="J4" s="2">
+        <f>IF(OR((I4="WATCH"),(H4&lt;0.5)),"REVIEW","OK")</f>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="4">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5">
+        <v>1310</v>
+      </c>
+      <c r="D5" s="18">
+        <v>0.18</v>
+      </c>
+      <c r="E5" s="4">
+        <v>16</v>
+      </c>
+      <c r="F5" s="5">
+        <f>ROUND((B5*C5),2)</f>
+      </c>
+      <c r="G5" s="5">
+        <f>ROUND((F5*(1-D5)),2)</f>
+      </c>
+      <c r="H5" s="14">
+        <f>IF((B5&gt;0),ROUND((E5/B5),4),0)</f>
+      </c>
+      <c r="I5" s="2">
+        <f>IF(OR((G5&gt;=5000),(H5&gt;=0.85)),"HIGH",IF((D5&gt;=0.15),"WATCH","STANDARD"))</f>
+      </c>
+      <c r="J5" s="2">
+        <f>IF(OR((I5="WATCH"),(H5&lt;0.5)),"REVIEW","OK")</f>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="F6" s="13">
+        <f>ROUND(SUM(F2:F5),2)</f>
+      </c>
+      <c r="G6" s="13">
+        <f>ROUND(SUM(G2:G5),2)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>